<commit_message>
feat(orna): enxuga linha ornamental (remove Aurora/Vespera/Serena)
Reflete o enxugamento da linha Orna feito no guia comercial:
- Remove os 3 modelos redundantes (Aurora, Vespera, Serena) das fontes
  de seed/referência, evitando que `npm run import` os recrie.
- EOS e Astrea já constavam na linha Versa em todo o código (import-versa,
  images.ts SEO, llms.txt, xlsx) e no snapshot do banco — nada a mover.

Produtos são renderizados do Payload CMS (DB), sem lista hard-coded; a
remoção efetiva no site é ação manual no admin, documentada em
docs/ORNA_SIMPLIFY.md.

- products-to-import.xlsx: remove 4 linhas de rascunho (Aurora Flangeado,
  Autora Engastado, Vespera, Serena)
- all_products.txt: remove as mesmas linhas do dump de referência (68->64)
- docs/ORNA_SIMPLIFY.md: runbook das ações no admin do Payload

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/products-to-import.xlsx
+++ b/products-to-import.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q80"/>
+  <dimension ref="A1:Q76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3052,7 +3052,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Poste Ornamental Aurora Flangeado</t>
+          <t>Poste Ornamental Harmonia Flangeado</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3095,7 +3095,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Porte Ornamental Autora Engastado</t>
+          <t>Poste Ornamental Harmonia Engastado</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3137,12 +3137,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Poste Ornamental Harmonia Flangeado</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>NBR 6323, NBR 14744, Garantia B&amp;B</t>
+          <t>Poste Ornamental Heliptica Engastado</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -3163,49 +3158,6 @@
         </is>
       </c>
       <c r="N39" t="inlineStr">
-        <is>
-          <t>Chumbador,_x000d_
-Janela de Inspeção,_x000d_
-Projeto de Poste Personalizado,_x000d_
-Pintura Eletrostática a pó, Galnanização a Fogo, _x000d_
-Projeto Iluminotécnico</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>NBR 6323 / NBR 14744</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Poste Ornamental Harmonia Engastado</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>NBR 6323, NBR 14744, Garantia B&amp;B</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>Vias Públicas,_x000d_
-Praças e Parques,_x000d_
-Condomínios, Estacionamentos, Aeroportos, Agro, City</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>Aço Carbono</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>3m a 15m</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr">
         <is>
           <t>Janela de Inspeção,_x000d_
 Projeto de Poste Personalizado,_x000d_
@@ -3213,6 +3165,35 @@
 Projeto Iluminotécnico</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>NBR 6323 / NBR 14744</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Poste Ornamental Heliptica Flangeado</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Vias Públicas,_x000d_
+Praças e Parques,_x000d_
+Condomínios, Estacionamentos, Aeroportos, Agro, City</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Aço Carbono</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>3m a 15m</t>
+        </is>
+      </c>
       <c r="O40" t="inlineStr">
         <is>
           <t>NBR 6323 / NBR 14744</t>
@@ -3222,7 +3203,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Poste Ornamental Heliptica Engastado</t>
+          <t>Poste Ornamental Aquila Engastado</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -3259,7 +3240,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Poste Ornamental Heliptica Flangeado</t>
+          <t>Poste Ornamental Aquila Flangeado</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -3288,7 +3269,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Poste Ornamental Aquila Engastado</t>
+          <t>Poste Ornamental Lyra</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -3308,14 +3289,6 @@
           <t>3m a 15m</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>Janela de Inspeção,_x000d_
-Projeto de Poste Personalizado,_x000d_
-Pintura Eletrostática a pó, Galnanização a Fogo, _x000d_
-Projeto Iluminotécnico</t>
-        </is>
-      </c>
       <c r="O43" t="inlineStr">
         <is>
           <t>NBR 6323 / NBR 14744</t>
@@ -3323,11 +3296,6 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Poste Ornamental Aquila Flangeado</t>
-        </is>
-      </c>
       <c r="J44" t="inlineStr">
         <is>
           <t>Vias Públicas,_x000d_
@@ -3354,7 +3322,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Poste Ornamental Lyra</t>
+          <t>Porte Ornamental Polaris</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -3407,7 +3375,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Porte Ornamental Polaris</t>
+          <t>Poste Ornamental Phoenix</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -3460,7 +3428,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Poste Ornamental Phoenix</t>
+          <t>Poste Ornamental Astra</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -3513,7 +3481,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Poste Ornamental Astra</t>
+          <t>Poste Ornamental Arcus</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -3566,7 +3534,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Poste Ornamental Arcus</t>
+          <t>Poste Ornamental Altair</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -3619,7 +3587,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Poste Ornamental Altair</t>
+          <t>Poste Ornamental Ignis</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -3672,7 +3640,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Poste Ornamental Ignis</t>
+          <t>Poste Ornamental Orionis</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3725,7 +3693,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Poste Ornamental Orionis</t>
+          <t>Poste Ornamental Aurion</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -3776,11 +3744,6 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Poste Ornamental Aurion</t>
-        </is>
-      </c>
       <c r="J61" t="inlineStr">
         <is>
           <t>Vias Públicas,_x000d_
@@ -3805,6 +3768,11 @@
       </c>
     </row>
     <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Poste Ornamental Aurum</t>
+        </is>
+      </c>
       <c r="J62" t="inlineStr">
         <is>
           <t>Vias Públicas,_x000d_
@@ -3829,11 +3797,6 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Poste Ornamental Vespera</t>
-        </is>
-      </c>
       <c r="J63" t="inlineStr">
         <is>
           <t>Vias Públicas,_x000d_
@@ -3858,6 +3821,11 @@
       </c>
     </row>
     <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Poste Ornamental Halo</t>
+        </is>
+      </c>
       <c r="J64" t="inlineStr">
         <is>
           <t>Vias Públicas,_x000d_
@@ -3882,11 +3850,6 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Poste Ornamental Aurum</t>
-        </is>
-      </c>
       <c r="J65" t="inlineStr">
         <is>
           <t>Vias Públicas,_x000d_
@@ -3911,6 +3874,11 @@
       </c>
     </row>
     <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Poste Ornamental Zéfiro</t>
+        </is>
+      </c>
       <c r="J66" t="inlineStr">
         <is>
           <t>Vias Públicas,_x000d_
@@ -3935,11 +3903,6 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Poste Ornamental Halo</t>
-        </is>
-      </c>
       <c r="J67" t="inlineStr">
         <is>
           <t>Vias Públicas,_x000d_
@@ -3964,6 +3927,11 @@
       </c>
     </row>
     <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Poste Ornamental Pyxis</t>
+        </is>
+      </c>
       <c r="J68" t="inlineStr">
         <is>
           <t>Vias Públicas,_x000d_
@@ -3988,11 +3956,6 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Poste Ornamental Zéfiro</t>
-        </is>
-      </c>
       <c r="J69" t="inlineStr">
         <is>
           <t>Vias Públicas,_x000d_
@@ -4017,6 +3980,11 @@
       </c>
     </row>
     <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Poste Ornamental Vela</t>
+        </is>
+      </c>
       <c r="J70" t="inlineStr">
         <is>
           <t>Vias Públicas,_x000d_
@@ -4041,11 +4009,6 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Poste Ornamental Pyxis</t>
-        </is>
-      </c>
       <c r="J71" t="inlineStr">
         <is>
           <t>Vias Públicas,_x000d_
@@ -4070,11 +4033,49 @@
       </c>
     </row>
     <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Poste Astrea</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>poste-ornamental-astrea</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>BB-VRS-ASTXX</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Versa</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Poste decorativo com estrutura ornamental ramificada, pensado para distribuir a luz de forma ampla. Solução com presença escultural para praças, acessos e áreas de convivência.</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>15 a 20 dias úteis</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>poste-astrea.png</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>NBR 6323, NBR 14744, Garantia B&amp;B</t>
+        </is>
+      </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Vias Públicas,_x000d_
-Praças e Parques,_x000d_
-Condomínios, Estacionamentos, Aeroportos, Agro, City</t>
+          <t>Praças, Acessos, Áreas de convivência, Condomínios, Fachadas</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -4084,7 +4085,12 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>3m a 15m</t>
+          <t>2m a 6m</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>Projeto Personalizado, Pintura Eletrostática, Projeto Iluminotécnico</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
@@ -4094,11 +4100,6 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Poste Ornamental Vela</t>
-        </is>
-      </c>
       <c r="J73" t="inlineStr">
         <is>
           <t>Vias Públicas,_x000d_
@@ -4149,238 +4150,94 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Poste Astrea</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>poste-ornamental-astrea</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>BB-VRS-ASTXX</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
+          <t>Poste Ornamental Atlas</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Vias Públicas,_x000d_
+Praças e Parques,_x000d_
+Condomínios, Estacionamentos, Aeroportos, Agro, City</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Aço Carbono</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>3m a 15m</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>NBR 6323 / NBR 14744</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Poste EOS</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>poste-ornamental-eos</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>BB-VRS-EOSXX</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
         <is>
           <t>Versa</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>Poste decorativo com estrutura ornamental ramificada, pensado para distribuir a luz de forma ampla. Solução com presença escultural para praças, acessos e áreas de convivência.</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Poste decorativo de globos com luz difusa e ornamental. Indicado para praças, jardins e áreas de convivência que pedem conforto visual e presença arquitetônica.</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
         <is>
           <t>15 a 20 dias úteis</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>poste-astrea.png</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>poste-eos.png</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
         <is>
           <t>NBR 6323, NBR 14744, Garantia B&amp;B</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>Praças, Acessos, Áreas de convivência, Condomínios, Fachadas</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>Aço Carbono</t>
-        </is>
-      </c>
-      <c r="L75" t="inlineStr">
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Praças, Jardins, Áreas de convivência, Condomínios, Fachadas</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Aço Carbono</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
         <is>
           <t>2m a 6m</t>
         </is>
       </c>
-      <c r="N75" t="inlineStr">
+      <c r="N76" t="inlineStr">
         <is>
           <t>Projeto Personalizado, Pintura Eletrostática, Projeto Iluminotécnico</t>
         </is>
       </c>
-      <c r="O75" t="inlineStr">
-        <is>
-          <t>NBR 6323 / NBR 14744</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>Vias Públicas,_x000d_
-Praças e Parques,_x000d_
-Condomínios, Estacionamentos, Aeroportos, Agro, City</t>
-        </is>
-      </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>Aço Carbono</t>
-        </is>
-      </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>3m a 15m</t>
-        </is>
-      </c>
       <c r="O76" t="inlineStr">
-        <is>
-          <t>NBR 6323 / NBR 14744</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Poste Ornamental Serena</t>
-        </is>
-      </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>Vias Públicas,_x000d_
-Praças e Parques,_x000d_
-Condomínios, Estacionamentos, Aeroportos, Agro, City</t>
-        </is>
-      </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>Aço Carbono</t>
-        </is>
-      </c>
-      <c r="L77" t="inlineStr">
-        <is>
-          <t>3m a 15m</t>
-        </is>
-      </c>
-      <c r="O77" t="inlineStr">
-        <is>
-          <t>NBR 6323 / NBR 14744</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>Vias Públicas,_x000d_
-Praças e Parques,_x000d_
-Condomínios, Estacionamentos, Aeroportos, Agro, City</t>
-        </is>
-      </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>Aço Carbono</t>
-        </is>
-      </c>
-      <c r="L78" t="inlineStr">
-        <is>
-          <t>3m a 15m</t>
-        </is>
-      </c>
-      <c r="O78" t="inlineStr">
-        <is>
-          <t>NBR 6323 / NBR 14744</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>Poste Ornamental Atlas</t>
-        </is>
-      </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>Vias Públicas,_x000d_
-Praças e Parques,_x000d_
-Condomínios, Estacionamentos, Aeroportos, Agro, City</t>
-        </is>
-      </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>Aço Carbono</t>
-        </is>
-      </c>
-      <c r="L79" t="inlineStr">
-        <is>
-          <t>3m a 15m</t>
-        </is>
-      </c>
-      <c r="O79" t="inlineStr">
-        <is>
-          <t>NBR 6323 / NBR 14744</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>Poste EOS</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>poste-ornamental-eos</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>BB-VRS-EOSXX</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Versa</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>Poste decorativo de globos com luz difusa e ornamental. Indicado para praças, jardins e áreas de convivência que pedem conforto visual e presença arquitetônica.</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>15 a 20 dias úteis</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>poste-eos.png</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>NBR 6323, NBR 14744, Garantia B&amp;B</t>
-        </is>
-      </c>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t>Praças, Jardins, Áreas de convivência, Condomínios, Fachadas</t>
-        </is>
-      </c>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>Aço Carbono</t>
-        </is>
-      </c>
-      <c r="L80" t="inlineStr">
-        <is>
-          <t>2m a 6m</t>
-        </is>
-      </c>
-      <c r="N80" t="inlineStr">
-        <is>
-          <t>Projeto Personalizado, Pintura Eletrostática, Projeto Iluminotécnico</t>
-        </is>
-      </c>
-      <c r="O80" t="inlineStr">
         <is>
           <t>NBR 6323 / NBR 14744</t>
         </is>

</xml_diff>